<commit_message>
Update Hess Flipper question database
</commit_message>
<xml_diff>
--- a/data/hess_flipper_questions.xlsx
+++ b/data/hess_flipper_questions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamsun/Documents/Codex/Hess消消乐/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB105D4A-4204-A74B-B554-E63785A565DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F334281-45BC-004A-AEB1-D3A59428AAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QUESTIONS" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="359">
   <si>
     <t>question_id</t>
   </si>
@@ -1220,6 +1220,154 @@
   </si>
   <si>
     <t>Required dp = max(highest dp among all Given delta_h values, 1 dp if scaling by a fraction produces a non-integer ΔH). If the division is exact and produces an integer, no extra decimal place is required. Round only the final answer.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>HF041</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>2 Al(s) + 3 Cl2(g) -&gt; 2 AlCl3(s)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>HF042</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>2 Al(s) + 6 HCl(aq) -&gt; 2 AlCl3(aq) + 3 H2(g)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>HCl(g) -&gt; HCl(aq)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>H2(g) + Cl2(g) -&gt; 2 HCl(g)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>AlCl3(s) -&gt; AlCl3(aq)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-1049</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-74.8</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-323</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>PbCl2(s) + Cl2(g) -&gt; PbCl4(l)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pb(s) + 2 Cl2(g) -&gt; PbCl4(l)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pb(s) + Cl2(g) -&gt; PbCl2(s)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-393</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-359</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>HF043</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hg2Cl2(s) -&gt; 2 Hg(l) + Cl2(g)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hg(l) + Cl2(g) -&gt; HgCl2(s)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hg(l) + HgCl2(s) -&gt; Hg2Cl2(s)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-224</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-41.2</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>HF044</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>SiO2(s) + 3 C(graphite) -&gt; SiC(s) + 2 CO(g)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Si(s) + O2(g) -&gt; SiO2(s)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Si(s) + C(graphite) -&gt; SiC(s)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-911</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-221</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-65.3</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>HF045</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>H2B4O7(s) + H2O(l) -&gt; 4 HBO2(aq)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>2 H3BO3(aq) -&gt; B2O3(s) + 3 H2O(l)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>H3BO3(aq) -&gt; HBO2(aq) + H2O(l)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>H2B4O7(s) -&gt; 2 B2O3(s) + H2O(l)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>14.4</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-0.02</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>17.3</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>-184.5</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -1569,7 +1717,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="QuestionsTable" displayName="QuestionsTable" ref="A1:D85" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="QuestionsTable" displayName="QuestionsTable" ref="A1:D83" totalsRowShown="0">
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="question_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="difficulty"/>
@@ -1581,7 +1729,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ReactionsTable" displayName="ReactionsTable" ref="A1:D315" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ReactionsTable" displayName="ReactionsTable" ref="A1:D299" totalsRowShown="0">
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="question_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="reaction_no" dataDxfId="0"/>
@@ -1787,7 +1935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1815,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>8</v>
+        <v>117</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>85</v>
@@ -1843,7 +1991,7 @@
         <v>59</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>92</v>
@@ -1955,7 +2103,7 @@
         <v>67</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>8</v>
+        <v>117</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>144</v>
@@ -1969,7 +2117,7 @@
         <v>68</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>117</v>
+        <v>8</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>150</v>
@@ -1997,7 +2145,7 @@
         <v>70</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>117</v>
+        <v>4</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>165</v>
@@ -2011,7 +2159,7 @@
         <v>71</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>117</v>
+        <v>4</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>173</v>
@@ -2025,7 +2173,7 @@
         <v>72</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>8</v>
+        <v>117</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>180</v>
@@ -2067,7 +2215,7 @@
         <v>75</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>117</v>
+        <v>8</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>194</v>
@@ -2137,7 +2285,7 @@
         <v>80</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>8</v>
+        <v>117</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>229</v>
@@ -2356,35 +2504,75 @@
         <v>260</v>
       </c>
     </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="9"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="9"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="9"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="9"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" s="9"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
+    <row r="41" spans="1:4" ht="15">
+      <c r="A41" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="15">
+      <c r="A42" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="15">
+      <c r="A43" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="15">
+      <c r="A44" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="15">
+      <c r="A45" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C45" t="s">
+        <v>351</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="9"/>
@@ -2609,10 +2797,10 @@
       <c r="D82" s="6"/>
     </row>
     <row r="83" spans="1:4">
-      <c r="A83" s="9"/>
-      <c r="B83" s="4"/>
-      <c r="C83" s="6"/>
-      <c r="D83" s="6"/>
+      <c r="A83" s="10"/>
+      <c r="B83" s="5"/>
+      <c r="C83" s="7"/>
+      <c r="D83" s="7"/>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="9"/>
@@ -2621,10 +2809,10 @@
       <c r="D84" s="6"/>
     </row>
     <row r="85" spans="1:4">
-      <c r="A85" s="10"/>
-      <c r="B85" s="5"/>
-      <c r="C85" s="7"/>
-      <c r="D85" s="7"/>
+      <c r="A85" s="9"/>
+      <c r="B85" s="4"/>
+      <c r="C85" s="6"/>
+      <c r="D85" s="6"/>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="9"/>
@@ -2855,28 +3043,16 @@
       <c r="D123" s="6"/>
     </row>
     <row r="124" spans="1:4">
-      <c r="A124" s="9"/>
-      <c r="B124" s="4"/>
-      <c r="C124" s="6"/>
-      <c r="D124" s="6"/>
-    </row>
-    <row r="125" spans="1:4">
-      <c r="A125" s="9"/>
-      <c r="B125" s="4"/>
-      <c r="C125" s="6"/>
-      <c r="D125" s="6"/>
-    </row>
-    <row r="126" spans="1:4">
-      <c r="A126" s="10"/>
-      <c r="B126" s="5"/>
-      <c r="C126" s="7"/>
-      <c r="D126" s="7"/>
+      <c r="A124" s="10"/>
+      <c r="B124" s="5"/>
+      <c r="C124" s="7"/>
+      <c r="D124" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="B2:B126" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>"Easy,Medium,Hard"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{89307292-35E8-0944-9102-EF8354EF6B3B}">
+      <formula1>"Easy,Medium,Hard,Extreme"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2888,7 +3064,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D998"/>
+  <dimension ref="A1:D982"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -4256,62 +4432,200 @@
       </c>
     </row>
     <row r="98" spans="1:4">
-      <c r="A98" s="10"/>
-      <c r="B98" s="24"/>
-      <c r="C98" s="7"/>
-      <c r="D98" s="12"/>
+      <c r="A98" t="s">
+        <v>322</v>
+      </c>
+      <c r="B98" s="25">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>325</v>
+      </c>
+      <c r="D98" s="13" t="s">
+        <v>329</v>
+      </c>
     </row>
     <row r="99" spans="1:4">
-      <c r="B99" s="25"/>
-      <c r="D99" s="13"/>
+      <c r="A99" t="s">
+        <v>322</v>
+      </c>
+      <c r="B99" s="25">
+        <v>2</v>
+      </c>
+      <c r="C99" t="s">
+        <v>326</v>
+      </c>
+      <c r="D99" s="13" t="s">
+        <v>330</v>
+      </c>
     </row>
     <row r="100" spans="1:4">
-      <c r="B100" s="25"/>
-      <c r="D100" s="13"/>
+      <c r="A100" t="s">
+        <v>322</v>
+      </c>
+      <c r="B100" s="25">
+        <v>3</v>
+      </c>
+      <c r="C100" t="s">
+        <v>327</v>
+      </c>
+      <c r="D100" s="13" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="101" spans="1:4">
-      <c r="B101" s="25"/>
-      <c r="D101" s="13"/>
+      <c r="A101" t="s">
+        <v>322</v>
+      </c>
+      <c r="B101" s="25">
+        <v>4</v>
+      </c>
+      <c r="C101" t="s">
+        <v>328</v>
+      </c>
+      <c r="D101" s="13" t="s">
+        <v>331</v>
+      </c>
     </row>
     <row r="102" spans="1:4">
-      <c r="B102" s="25"/>
-      <c r="D102" s="13"/>
+      <c r="A102" t="s">
+        <v>324</v>
+      </c>
+      <c r="B102" s="25">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>333</v>
+      </c>
+      <c r="D102" s="13" t="s">
+        <v>335</v>
+      </c>
     </row>
     <row r="103" spans="1:4">
-      <c r="B103" s="25"/>
-      <c r="D103" s="13"/>
+      <c r="A103" t="s">
+        <v>324</v>
+      </c>
+      <c r="B103" s="25">
+        <v>2</v>
+      </c>
+      <c r="C103" t="s">
+        <v>334</v>
+      </c>
+      <c r="D103" s="13" t="s">
+        <v>336</v>
+      </c>
     </row>
     <row r="104" spans="1:4">
-      <c r="B104" s="25"/>
-      <c r="D104" s="13"/>
+      <c r="A104" t="s">
+        <v>337</v>
+      </c>
+      <c r="B104" s="25">
+        <v>1</v>
+      </c>
+      <c r="C104" t="s">
+        <v>339</v>
+      </c>
+      <c r="D104" s="13" t="s">
+        <v>341</v>
+      </c>
     </row>
     <row r="105" spans="1:4">
-      <c r="B105" s="25"/>
-      <c r="D105" s="13"/>
+      <c r="A105" t="s">
+        <v>337</v>
+      </c>
+      <c r="B105" s="25">
+        <v>2</v>
+      </c>
+      <c r="C105" t="s">
+        <v>340</v>
+      </c>
+      <c r="D105" s="13" t="s">
+        <v>342</v>
+      </c>
     </row>
     <row r="106" spans="1:4">
-      <c r="B106" s="25"/>
-      <c r="D106" s="13"/>
+      <c r="A106" t="s">
+        <v>343</v>
+      </c>
+      <c r="B106" s="25">
+        <v>1</v>
+      </c>
+      <c r="C106" t="s">
+        <v>345</v>
+      </c>
+      <c r="D106" s="13" t="s">
+        <v>347</v>
+      </c>
     </row>
     <row r="107" spans="1:4">
-      <c r="B107" s="25"/>
-      <c r="D107" s="13"/>
+      <c r="A107" t="s">
+        <v>343</v>
+      </c>
+      <c r="B107" s="25">
+        <v>2</v>
+      </c>
+      <c r="C107" t="s">
+        <v>249</v>
+      </c>
+      <c r="D107" s="13" t="s">
+        <v>348</v>
+      </c>
     </row>
     <row r="108" spans="1:4">
-      <c r="B108" s="25"/>
-      <c r="D108" s="13"/>
+      <c r="A108" t="s">
+        <v>343</v>
+      </c>
+      <c r="B108" s="25">
+        <v>3</v>
+      </c>
+      <c r="C108" t="s">
+        <v>346</v>
+      </c>
+      <c r="D108" s="13" t="s">
+        <v>349</v>
+      </c>
     </row>
     <row r="109" spans="1:4">
-      <c r="B109" s="25"/>
-      <c r="D109" s="13"/>
+      <c r="A109" t="s">
+        <v>350</v>
+      </c>
+      <c r="B109" s="25">
+        <v>1</v>
+      </c>
+      <c r="C109" t="s">
+        <v>352</v>
+      </c>
+      <c r="D109" s="13" t="s">
+        <v>355</v>
+      </c>
     </row>
     <row r="110" spans="1:4">
-      <c r="B110" s="25"/>
-      <c r="D110" s="13"/>
+      <c r="A110" t="s">
+        <v>350</v>
+      </c>
+      <c r="B110" s="25">
+        <v>2</v>
+      </c>
+      <c r="C110" t="s">
+        <v>353</v>
+      </c>
+      <c r="D110" s="13" t="s">
+        <v>356</v>
+      </c>
     </row>
     <row r="111" spans="1:4">
-      <c r="B111" s="25"/>
-      <c r="D111" s="13"/>
+      <c r="A111" t="s">
+        <v>350</v>
+      </c>
+      <c r="B111" s="25">
+        <v>3</v>
+      </c>
+      <c r="C111" t="s">
+        <v>354</v>
+      </c>
+      <c r="D111" s="13" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="112" spans="1:4">
       <c r="B112" s="25"/>
@@ -5066,82 +5380,66 @@
       <c r="D299" s="13"/>
     </row>
     <row r="300" spans="2:4">
-      <c r="B300" s="25"/>
       <c r="D300" s="13"/>
     </row>
     <row r="301" spans="2:4">
-      <c r="B301" s="25"/>
       <c r="D301" s="13"/>
     </row>
     <row r="302" spans="2:4">
-      <c r="B302" s="25"/>
       <c r="D302" s="13"/>
     </row>
     <row r="303" spans="2:4">
-      <c r="B303" s="25"/>
       <c r="D303" s="13"/>
     </row>
     <row r="304" spans="2:4">
-      <c r="B304" s="25"/>
       <c r="D304" s="13"/>
     </row>
-    <row r="305" spans="2:4">
-      <c r="B305" s="25"/>
+    <row r="305" spans="4:4">
       <c r="D305" s="13"/>
     </row>
-    <row r="306" spans="2:4">
-      <c r="B306" s="25"/>
+    <row r="306" spans="4:4">
       <c r="D306" s="13"/>
     </row>
-    <row r="307" spans="2:4">
-      <c r="B307" s="25"/>
+    <row r="307" spans="4:4">
       <c r="D307" s="13"/>
     </row>
-    <row r="308" spans="2:4">
-      <c r="B308" s="25"/>
+    <row r="308" spans="4:4">
       <c r="D308" s="13"/>
     </row>
-    <row r="309" spans="2:4">
-      <c r="B309" s="25"/>
+    <row r="309" spans="4:4">
       <c r="D309" s="13"/>
     </row>
-    <row r="310" spans="2:4">
-      <c r="B310" s="25"/>
+    <row r="310" spans="4:4">
       <c r="D310" s="13"/>
     </row>
-    <row r="311" spans="2:4">
-      <c r="B311" s="25"/>
+    <row r="311" spans="4:4">
       <c r="D311" s="13"/>
     </row>
-    <row r="312" spans="2:4">
-      <c r="B312" s="25"/>
+    <row r="312" spans="4:4">
       <c r="D312" s="13"/>
     </row>
-    <row r="313" spans="2:4">
-      <c r="B313" s="25"/>
+    <row r="313" spans="4:4">
       <c r="D313" s="13"/>
     </row>
-    <row r="314" spans="2:4">
-      <c r="B314" s="25"/>
+    <row r="314" spans="4:4">
       <c r="D314" s="13"/>
     </row>
-    <row r="315" spans="2:4">
-      <c r="B315" s="25"/>
+    <row r="315" spans="4:4">
       <c r="D315" s="13"/>
     </row>
-    <row r="316" spans="2:4">
+    <row r="316" spans="4:4">
       <c r="D316" s="13"/>
     </row>
-    <row r="317" spans="2:4">
+    <row r="317" spans="4:4">
       <c r="D317" s="13"/>
     </row>
-    <row r="318" spans="2:4">
+    <row r="318" spans="4:4">
       <c r="D318" s="13"/>
     </row>
-    <row r="319" spans="2:4">
+    <row r="319" spans="4:4">
       <c r="D319" s="13"/>
     </row>
-    <row r="320" spans="2:4">
+    <row r="320" spans="4:4">
       <c r="D320" s="13"/>
     </row>
     <row r="321" spans="4:4">
@@ -7129,54 +7427,6 @@
     </row>
     <row r="982" spans="4:4">
       <c r="D982" s="13"/>
-    </row>
-    <row r="983" spans="4:4">
-      <c r="D983" s="13"/>
-    </row>
-    <row r="984" spans="4:4">
-      <c r="D984" s="13"/>
-    </row>
-    <row r="985" spans="4:4">
-      <c r="D985" s="13"/>
-    </row>
-    <row r="986" spans="4:4">
-      <c r="D986" s="13"/>
-    </row>
-    <row r="987" spans="4:4">
-      <c r="D987" s="13"/>
-    </row>
-    <row r="988" spans="4:4">
-      <c r="D988" s="13"/>
-    </row>
-    <row r="989" spans="4:4">
-      <c r="D989" s="13"/>
-    </row>
-    <row r="990" spans="4:4">
-      <c r="D990" s="13"/>
-    </row>
-    <row r="991" spans="4:4">
-      <c r="D991" s="13"/>
-    </row>
-    <row r="992" spans="4:4">
-      <c r="D992" s="13"/>
-    </row>
-    <row r="993" spans="4:4">
-      <c r="D993" s="13"/>
-    </row>
-    <row r="994" spans="4:4">
-      <c r="D994" s="13"/>
-    </row>
-    <row r="995" spans="4:4">
-      <c r="D995" s="13"/>
-    </row>
-    <row r="996" spans="4:4">
-      <c r="D996" s="13"/>
-    </row>
-    <row r="997" spans="4:4">
-      <c r="D997" s="13"/>
-    </row>
-    <row r="998" spans="4:4">
-      <c r="D998" s="13"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>

</xml_diff>